<commit_message>
Ratings are being picked and excel sheet is updating
</commit_message>
<xml_diff>
--- a/Reports/CarWashServices.xlsx
+++ b/Reports/CarWashServices.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>S.No</t>
   </si>
@@ -32,7 +32,7 @@
     <t>07942548952</t>
   </si>
   <si>
-    <t>N/A</t>
+    <t>4.7</t>
   </si>
   <si>
     <t>Car Washing Services At Home</t>
@@ -41,10 +41,16 @@
     <t>07942666907</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>Car Washing Service</t>
   </si>
   <si>
     <t>08047812127</t>
+  </si>
+  <si>
+    <t>3</t>
   </si>
 </sst>
 </file>
@@ -154,7 +160,7 @@
         <v>8</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -162,13 +168,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Allure auto-opening, final version
</commit_message>
<xml_diff>
--- a/Reports/CarWashServices.xlsx
+++ b/Reports/CarWashServices.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>S.No</t>
   </si>
@@ -26,7 +26,7 @@
     <t>Rating</t>
   </si>
   <si>
-    <t>Doorstep Car Wash Service</t>
+    <t>Car Washing Service</t>
   </si>
   <si>
     <t>07942548952</t>
@@ -44,9 +44,6 @@
     <t>5</t>
   </si>
   <si>
-    <t>Car Washing Service</t>
-  </si>
-  <si>
     <t>08047812127</t>
   </si>
   <si>
@@ -58,7 +55,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -66,29 +63,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="9"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="darkGray"/>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="18"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="18"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -103,9 +84,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="true" applyFill="true"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -115,23 +95,23 @@
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="5.31640625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="5.18359375" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="28.39453125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="14.8671875" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="6.90625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="14.58984375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="6.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="1">
+      <c r="A1" t="s" s="0">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="1">
+      <c r="B1" t="s" s="0">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="1">
+      <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="1">
+      <c r="D1" t="s" s="0">
         <v>3</v>
       </c>
     </row>
@@ -168,13 +148,13 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="D4" t="s" s="0">
         <v>11</v>
-      </c>
-      <c r="D4" t="s" s="0">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>